<commit_message>
update xlsx 2026-07-09 03:56
</commit_message>
<xml_diff>
--- a/EF成人英语_私信数据_2026-06.xlsx
+++ b/EF成人英语_私信数据_2026-06.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z6"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -435,18 +435,6 @@
     <col width="21" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="21" customWidth="1" min="18" max="18"/>
-    <col width="9" customWidth="1" min="19" max="19"/>
-    <col width="9" customWidth="1" min="20" max="20"/>
-    <col width="8" customWidth="1" min="21" max="21"/>
-    <col width="20" customWidth="1" min="22" max="22"/>
-    <col width="21" customWidth="1" min="23" max="23"/>
-    <col width="21" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="22" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -520,66 +508,6 @@
           <t>CTR</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>15s首响率</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>30s回复率</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>1min回复率</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>平均回复时长(分)-新</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>私信咨询数</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>私信开口数</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>私信留资数</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>进线开口率</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>开口留资率</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>进线留资率</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>私信留资成本</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>CTR</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -624,42 +552,6 @@
       <c r="N2" t="n">
         <v>0.02747895678192049</v>
       </c>
-      <c r="O2" t="n">
-        <v>0.9607867702330243</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.9946624803767661</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.9959183673469387</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1.682817155402227</v>
-      </c>
-      <c r="S2" t="n">
-        <v>24771</v>
-      </c>
-      <c r="T2" t="n">
-        <v>18416</v>
-      </c>
-      <c r="U2" t="n">
-        <v>8350</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0.7434500020184893</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.4534100781928758</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0.3370877235476969</v>
-      </c>
-      <c r="Y2" t="n">
-        <v>877.7305065868262</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0.02747895678192049</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -708,42 +600,6 @@
       <c r="N3" t="n">
         <v>0.03978702222666533</v>
       </c>
-      <c r="O3" t="n">
-        <v>0.9649191959006701</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.9877358490566037</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.994811320754717</v>
-      </c>
-      <c r="R3" t="n">
-        <v>17.28756868131868</v>
-      </c>
-      <c r="S3" t="n">
-        <v>2536</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1491</v>
-      </c>
-      <c r="U3" t="n">
-        <v>627</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.5879337539432177</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.420523138832998</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.2472397476340694</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>1145.495901116427</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0.03978702222666533</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -792,42 +648,6 @@
       <c r="N4" t="n">
         <v>0.02385594407535814</v>
       </c>
-      <c r="O4" t="n">
-        <v>0.9646424721523535</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0.9980151156576837</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0.9981677990686312</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0.1641834759576202</v>
-      </c>
-      <c r="S4" t="n">
-        <v>14507</v>
-      </c>
-      <c r="T4" t="n">
-        <v>10847</v>
-      </c>
-      <c r="U4" t="n">
-        <v>4929</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0.7477080030330185</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0.4544113579791648</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0.3397670090301234</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>813.9730594441064</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0.02385594407535814</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -876,42 +696,6 @@
       <c r="N5" t="n">
         <v>0.02868833736936087</v>
       </c>
-      <c r="O5" t="n">
-        <v>0.9529553679131484</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0.9967436352871522</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0.9972370238800079</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0.1385955370974653</v>
-      </c>
-      <c r="S5" t="n">
-        <v>7693</v>
-      </c>
-      <c r="T5" t="n">
-        <v>6046</v>
-      </c>
-      <c r="U5" t="n">
-        <v>2776</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0.785909268165865</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0.4591465431690374</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0.3608475237228649</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>933.3815814121034</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0.02868833736936087</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -958,42 +742,6 @@
         <v>426.8511111111113</v>
       </c>
       <c r="N6" t="n">
-        <v>0.02602266180142116</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0.7878787878787878</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0.5984251968503937</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0.6771653543307087</v>
-      </c>
-      <c r="R6" t="n">
-        <v>13.1609756097561</v>
-      </c>
-      <c r="S6" t="n">
-        <v>35</v>
-      </c>
-      <c r="T6" t="n">
-        <v>32</v>
-      </c>
-      <c r="U6" t="n">
-        <v>18</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0.9142857142857143</v>
-      </c>
-      <c r="W6" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="X6" t="n">
-        <v>0.5142857142857142</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>426.8511111111113</v>
-      </c>
-      <c r="Z6" t="n">
         <v>0.02602266180142116</v>
       </c>
     </row>
@@ -1008,24 +756,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:O6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="19" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1036,269 +784,318 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>15s首响率</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>30s回复率</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>1min回复率</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>平均回复时长(分)-新</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>私信咨询数</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>私信开口数</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>私信留资数</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>进线开口率</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>开口留资率</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>进线留资率</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>私信留资成本</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>曝光量</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>点击量</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>私信开口数</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>私信咨询数</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>私信留资数</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>CTR</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>私信留资成本</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>进线开口率</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>开口留资率</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>进线留资率</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>15s首响率</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>30s回复率</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>1min回复率</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>平均回复时长(分)-新</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>EF成人英语课程咨询 - 小F</t>
+          <t>总计</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>21900328</v>
+        <v>0.9594473245992577</v>
       </c>
       <c r="C2" t="n">
-        <v>522453</v>
+        <v>0.9957793704723732</v>
       </c>
       <c r="D2" t="n">
-        <v>10847</v>
+        <v>0.9967397855414215</v>
       </c>
       <c r="E2" t="n">
-        <v>14507</v>
+        <v>1.457738495253085</v>
       </c>
       <c r="F2" t="n">
-        <v>4929</v>
+        <v>23122</v>
       </c>
       <c r="G2" t="n">
-        <v>0.02385594407535814</v>
+        <v>17009</v>
       </c>
       <c r="H2" t="n">
-        <v>813.973059444106</v>
+        <v>7971</v>
       </c>
       <c r="I2" t="n">
-        <v>0.7477080030330185</v>
+        <v>0.735619756076464</v>
       </c>
       <c r="J2" t="n">
-        <v>0.4544113579791648</v>
+        <v>0.4686342524545828</v>
       </c>
       <c r="K2" t="n">
-        <v>0.3397670090301234</v>
+        <v>0.3447366144797163</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9646424721523535</v>
+        <v>766.9640544067175</v>
       </c>
       <c r="M2" t="n">
-        <v>0.9980151156576837</v>
+        <v>0.02543034129906833</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9981677990686312</v>
+        <v>34257228</v>
       </c>
       <c r="O2" t="n">
-        <v>0.1641834759576202</v>
+        <v>871173</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>EF成人英语课程咨询 - 小E</t>
+          <t>EF成人英语课程咨询 - 小F</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10075025</v>
+        <v>0.9646424721523535</v>
       </c>
       <c r="C3" t="n">
-        <v>264338</v>
+        <v>0.9980151156576837</v>
       </c>
       <c r="D3" t="n">
-        <v>4862</v>
+        <v>0.9981677990686312</v>
       </c>
       <c r="E3" t="n">
-        <v>6284</v>
+        <v>0.1641834759576202</v>
       </c>
       <c r="F3" t="n">
-        <v>2397</v>
+        <v>14507</v>
       </c>
       <c r="G3" t="n">
-        <v>0.02623695722839398</v>
+        <v>10847</v>
       </c>
       <c r="H3" t="n">
-        <v>676.8194817171241</v>
+        <v>4929</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7737110120942076</v>
+        <v>0.7477080030330185</v>
       </c>
       <c r="J3" t="n">
-        <v>0.493006993006993</v>
+        <v>0.4544113579791648</v>
       </c>
       <c r="K3" t="n">
-        <v>0.3814449395289625</v>
+        <v>0.3397670090301234</v>
       </c>
       <c r="L3" t="n">
-        <v>0.9475661548513558</v>
+        <v>813.973059444106</v>
       </c>
       <c r="M3" t="n">
-        <v>0.9963695543314972</v>
+        <v>0.02385594407535814</v>
       </c>
       <c r="N3" t="n">
-        <v>0.9969954932398598</v>
+        <v>21900328</v>
       </c>
       <c r="O3" t="n">
-        <v>0.1622841132438423</v>
+        <v>522453</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>EF成人英语培训</t>
+          <t>EF成人英语课程咨询 - 小E</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2261047</v>
+        <v>0.9475661548513558</v>
       </c>
       <c r="C4" t="n">
-        <v>83840</v>
+        <v>0.9963695543314972</v>
       </c>
       <c r="D4" t="n">
-        <v>1268</v>
+        <v>0.9969954932398598</v>
       </c>
       <c r="E4" t="n">
-        <v>2296</v>
+        <v>0.1622841132438423</v>
       </c>
       <c r="F4" t="n">
-        <v>627</v>
+        <v>6284</v>
       </c>
       <c r="G4" t="n">
-        <v>0.03708016684305988</v>
+        <v>4862</v>
       </c>
       <c r="H4" t="n">
-        <v>751.798484848485</v>
+        <v>2397</v>
       </c>
       <c r="I4" t="n">
-        <v>0.5522648083623694</v>
+        <v>0.7737110120942076</v>
       </c>
       <c r="J4" t="n">
-        <v>0.4944794952681388</v>
+        <v>0.493006993006993</v>
       </c>
       <c r="K4" t="n">
-        <v>0.2730836236933798</v>
+        <v>0.3814449395289625</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9617557583659279</v>
+        <v>676.8194817171241</v>
       </c>
       <c r="M4" t="n">
-        <v>0.9860950173812283</v>
+        <v>0.02623695722839398</v>
       </c>
       <c r="N4" t="n">
-        <v>0.9918887601390498</v>
+        <v>10075025</v>
       </c>
       <c r="O4" t="n">
-        <v>17.19526760563381</v>
+        <v>264338</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>EF成人英语培训</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.9617557583659279</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.9860950173812283</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.9918887601390498</v>
+      </c>
+      <c r="E5" t="n">
+        <v>17.19526760563381</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2296</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1268</v>
+      </c>
+      <c r="H5" t="n">
+        <v>627</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.5522648083623694</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.4944794952681388</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.2730836236933798</v>
+      </c>
+      <c r="L5" t="n">
+        <v>751.798484848485</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0.03708016684305988</v>
+      </c>
+      <c r="N5" t="n">
+        <v>2261047</v>
+      </c>
+      <c r="O5" t="n">
+        <v>83840</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>EF成人英语广东中心</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B6" t="n">
+        <v>0.7878787878787878</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.5984251968503937</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.6771653543307087</v>
+      </c>
+      <c r="E6" t="n">
+        <v>13.1609756097561</v>
+      </c>
+      <c r="F6" t="n">
+        <v>35</v>
+      </c>
+      <c r="G6" t="n">
+        <v>32</v>
+      </c>
+      <c r="H6" t="n">
+        <v>18</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.9142857142857143</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.5142857142857142</v>
+      </c>
+      <c r="L6" t="n">
+        <v>426.8511111111112</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0.02602266180142116</v>
+      </c>
+      <c r="N6" t="n">
         <v>20828</v>
       </c>
-      <c r="C5" t="n">
+      <c r="O6" t="n">
         <v>542</v>
-      </c>
-      <c r="D5" t="n">
-        <v>32</v>
-      </c>
-      <c r="E5" t="n">
-        <v>35</v>
-      </c>
-      <c r="F5" t="n">
-        <v>18</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.02602266180142116</v>
-      </c>
-      <c r="H5" t="n">
-        <v>426.8511111111112</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0.9142857142857143</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.5625</v>
-      </c>
-      <c r="K5" t="n">
-        <v>0.5142857142857142</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.7878787878787878</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0.5984251968503937</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0.6771653543307087</v>
-      </c>
-      <c r="O5" t="n">
-        <v>13.1609756097561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>